<commit_message>
first round of feedback
</commit_message>
<xml_diff>
--- a/backend/hutko_shop.xlsx
+++ b/backend/hutko_shop.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
@@ -150,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -181,6 +181,7 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -555,30 +556,30 @@
   <dimension ref="B1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="4" customWidth="1" style="17" min="2" max="2"/>
-    <col width="18" customWidth="1" style="17" min="3" max="5"/>
-    <col width="12" customWidth="1" style="17" min="6" max="6"/>
-    <col width="40" customWidth="1" style="17" min="7" max="9"/>
-    <col width="10" customWidth="1" style="17" min="10" max="12"/>
-    <col width="22" customWidth="1" style="17" min="13" max="14"/>
-    <col width="8" customWidth="1" style="17" min="15" max="15"/>
+    <col width="4" customWidth="1" style="18" min="2" max="2"/>
+    <col width="18" customWidth="1" style="18" min="3" max="5"/>
+    <col width="12" customWidth="1" style="18" min="6" max="6"/>
+    <col width="40" customWidth="1" style="18" min="7" max="9"/>
+    <col width="10" customWidth="1" style="18" min="10" max="12"/>
+    <col width="22" customWidth="1" style="18" min="13" max="14"/>
+    <col width="8" customWidth="1" style="18" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.4" customHeight="1" s="17">
-      <c r="B1" s="16" t="inlineStr">
+    <row r="1" ht="17.4" customHeight="1" s="18">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>🛒  HUTKO Kitchen — Product Catalogue</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="18" t="inlineStr">
+      <c r="B2" s="19" t="inlineStr">
         <is>
           <t>Edit this sheet to update the shop. photo_file = filename in assets/ folder. dietary = comma-separated tags.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1" s="17">
+    <row r="4" ht="30" customHeight="1" s="18">
       <c r="B4" s="1" t="inlineStr">
         <is>
           <t>id</t>
@@ -650,7 +651,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="40.05" customHeight="1" s="17">
+    <row r="5" ht="40.05" customHeight="1" s="18">
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>syrnyky</t>
@@ -716,7 +717,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="40.05" customHeight="1" s="17">
+    <row r="6" ht="40.05" customHeight="1" s="18">
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>chicken</t>
@@ -786,7 +787,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="40.05" customHeight="1" s="17">
+    <row r="7" ht="40.05" customHeight="1" s="18">
       <c r="B7" s="2" t="inlineStr">
         <is>
           <t>borscht</t>
@@ -852,7 +853,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="40.05" customHeight="1" s="17">
+    <row r="8" ht="40.05" customHeight="1" s="18">
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t>solyanka</t>
@@ -918,7 +919,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="40.05" customHeight="1" s="17">
+    <row r="9" ht="40.05" customHeight="1" s="18">
       <c r="B9" s="2" t="inlineStr">
         <is>
           <t>shakshuka</t>
@@ -988,7 +989,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="40.05" customHeight="1" s="17">
+    <row r="10" ht="40.05" customHeight="1" s="18">
       <c r="B10" s="3" t="inlineStr">
         <is>
           <t>zrazy</t>
@@ -1055,13 +1056,13 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>📦  PRODUCT VARIANTS (sizes &amp; prices)</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="52.8" customHeight="1" s="17">
+    <row r="13" ht="52.8" customHeight="1" s="18">
       <c r="B13" s="4" t="inlineStr">
         <is>
           <t>product_id</t>
@@ -1328,7 +1329,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;"Calibri"&amp;10 &amp;KFF0000_x000d_# C2-Vertrouwelijk</oddFooter>
+    <oddFooter>&amp;C&amp;"Calibri"&amp;10 &amp;KFF0000_x000d_# C2-Vertrouwelijk_x000d_&amp;1#&amp;"Calibri"&amp;10 &amp;K008000 C0-Openbaar</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1346,32 +1347,32 @@
   <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="4" customWidth="1" style="17" min="2" max="2"/>
-    <col width="20" customWidth="1" style="17" min="3" max="5"/>
-    <col width="10" customWidth="1" style="17" min="6" max="6"/>
-    <col width="45" customWidth="1" style="17" min="7" max="7"/>
-    <col width="12" customWidth="1" style="17" min="8" max="9"/>
-    <col width="25" customWidth="1" style="17" min="10" max="10"/>
-    <col width="15" customWidth="1" style="17" min="11" max="11"/>
-    <col width="8" customWidth="1" style="17" min="12" max="12"/>
+    <col width="4" customWidth="1" style="18" min="2" max="2"/>
+    <col width="20" customWidth="1" style="18" min="3" max="5"/>
+    <col width="10" customWidth="1" style="18" min="6" max="6"/>
+    <col width="45" customWidth="1" style="18" min="7" max="7"/>
+    <col width="12" customWidth="1" style="18" min="8" max="9"/>
+    <col width="25" customWidth="1" style="18" min="10" max="10"/>
+    <col width="15" customWidth="1" style="18" min="11" max="11"/>
+    <col width="8" customWidth="1" style="18" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.4" customHeight="1" s="17">
-      <c r="B1" s="16" t="inlineStr">
+    <row r="1" ht="17.4" customHeight="1" s="18">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>🎁  HUTKO Kitchen — Bundles &amp; Packs</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="18" t="inlineStr">
+      <c r="B2" s="19" t="inlineStr">
         <is>
           <t>items = product_id:qty,product_id:qty format. discount_price overrides calculated price.</t>
         </is>
       </c>
     </row>
     <row r="3"/>
-    <row r="4" ht="30" customHeight="1" s="17">
+    <row r="4" ht="30" customHeight="1" s="18">
       <c r="B4" s="1" t="inlineStr">
         <is>
           <t>id</t>
@@ -1428,7 +1429,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="45" customHeight="1" s="17">
+    <row r="5" ht="45" customHeight="1" s="18">
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>pack-s1</t>
@@ -1467,7 +1468,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>assets/hf_20260308_101724_332ed7b633c04af6be57da9339c4624d.jpeg</t>
+          <t>assets/IMG_4178.JPEG</t>
         </is>
       </c>
       <c r="K5" s="2" t="n"/>
@@ -1477,7 +1478,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1" s="17">
+    <row r="6" ht="45" customHeight="1" s="18">
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>pack-s2</t>
@@ -1516,7 +1517,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>assets/hf_20260308_101754_0817f1096b73448d87eb3531e411155b.png</t>
+          <t>assets/IMG_4176.JPEG</t>
         </is>
       </c>
       <c r="K6" s="3" t="n"/>
@@ -1526,7 +1527,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1" s="17">
+    <row r="7" ht="45" customHeight="1" s="18">
       <c r="B7" s="2" t="inlineStr">
         <is>
           <t>pack-m1</t>
@@ -1565,7 +1566,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>assets/hf_20260308_102232_0b1e6e0deade4ce2934cc28ee2635165.png</t>
+          <t>assets/IMG_4180.JPEG</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1579,7 +1580,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="45" customHeight="1" s="17">
+    <row r="8" ht="45" customHeight="1" s="18">
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t>pack-m2</t>
@@ -1618,7 +1619,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>assets/hf_20260308_102519_c328da66a77a47afaa22022eb4f842f1.png</t>
+          <t>assets/IMG_4180.JPEG</t>
         </is>
       </c>
       <c r="K8" s="3" t="n"/>
@@ -1628,7 +1629,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="45" customHeight="1" s="17">
+    <row r="9" ht="45" customHeight="1" s="18">
       <c r="B9" s="2" t="inlineStr">
         <is>
           <t>pack-l1</t>
@@ -1667,7 +1668,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>assets/hf_20260308_102551_7e65581e179545a7a46d6504b44e7e7b.png</t>
+          <t>assets/IMG_4156.PNG</t>
         </is>
       </c>
       <c r="K9" s="2" t="n"/>
@@ -1677,7 +1678,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="45" customHeight="1" s="17">
+    <row r="10" ht="45" customHeight="1" s="18">
       <c r="B10" s="3" t="inlineStr">
         <is>
           <t>pack-l2</t>
@@ -1716,7 +1717,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>assets/hf_20260308_103416_d2ba00b8715544dfb6886f8a1950d1c6.jpeg</t>
+          <t>assets/IMG_4156.PNG</t>
         </is>
       </c>
       <c r="K10" s="3" t="n"/>
@@ -1734,7 +1735,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;"Calibri"&amp;10 &amp;KFF0000_x000d_# C2-Vertrouwelijk</oddFooter>
+    <oddFooter>&amp;C&amp;"Calibri"&amp;10 &amp;KFF0000_x000d_# C2-Vertrouwelijk_x000d_&amp;1#&amp;"Calibri"&amp;10 &amp;K008000 C0-Openbaar</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1752,12 +1753,12 @@
   <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="75" customWidth="1" style="17" min="1" max="1"/>
-    <col width="25" customWidth="1" style="17" min="2" max="2"/>
-    <col width="60" customWidth="1" style="17" min="3" max="3"/>
+    <col width="75" customWidth="1" style="18" min="1" max="1"/>
+    <col width="25" customWidth="1" style="18" min="2" max="2"/>
+    <col width="60" customWidth="1" style="18" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.6" customHeight="1" s="17">
+    <row r="1" ht="15.6" customHeight="1" s="18">
       <c r="A1" s="7" t="inlineStr">
         <is>
           <t>📖  HOW TO USE THIS FILE</t>
@@ -1856,7 +1857,7 @@
     <row r="17">
       <c r="A17" s="8" t="n"/>
     </row>
-    <row r="18" ht="15.6" customHeight="1" s="17">
+    <row r="18" ht="15.6" customHeight="1" s="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
           <t>⚠️  AFTER EDITING:</t>
@@ -1888,7 +1889,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;"Calibri"&amp;10 &amp;KFF0000_x000d_# C2-Vertrouwelijk</oddFooter>
+    <oddFooter>&amp;C&amp;"Calibri"&amp;10 &amp;KFF0000_x000d_# C2-Vertrouwelijk_x000d_&amp;1#&amp;"Calibri"&amp;10 &amp;K008000 C0-Openbaar</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1907,27 +1908,27 @@
   <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="12" customWidth="1" style="17" min="1" max="1"/>
-    <col width="16" customWidth="1" style="17" min="2" max="2"/>
-    <col width="24" customWidth="1" style="17" min="3" max="3"/>
-    <col width="55" customWidth="1" style="17" min="4" max="4"/>
+    <col width="12" customWidth="1" style="18" min="1" max="1"/>
+    <col width="16" customWidth="1" style="18" min="2" max="2"/>
+    <col width="24" customWidth="1" style="18" min="3" max="3"/>
+    <col width="55" customWidth="1" style="18" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="17">
-      <c r="A1" s="20" t="inlineStr">
+    <row r="1" ht="18" customHeight="1" s="18">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>🖼️  HUTKO Kitchen — Image Manager</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>Change photo_file values below to update images on the website. Use relative paths from the frontend folder (e.g. assets/products/syrnyky.png).</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="6" customHeight="1" s="17"/>
+    <row r="3" ht="6" customHeight="1" s="18"/>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -2222,7 +2223,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;"Calibri"&amp;10 &amp;KFF0000_x000d_# C2-Vertrouwelijk</oddFooter>
+    <oddFooter>&amp;C&amp;"Calibri"&amp;10 &amp;KFF0000_x000d_# C2-Vertrouwelijk_x000d_&amp;1#&amp;"Calibri"&amp;10 &amp;K008000 C0-Openbaar</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2241,26 +2242,26 @@
   <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="22" customWidth="1" style="17" min="1" max="1"/>
-    <col width="38" customWidth="1" style="17" min="2" max="2"/>
-    <col width="45" customWidth="1" style="17" min="3" max="3"/>
+    <col width="22" customWidth="1" style="18" min="1" max="1"/>
+    <col width="38" customWidth="1" style="18" min="2" max="2"/>
+    <col width="45" customWidth="1" style="18" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="17">
-      <c r="A1" s="20" t="inlineStr">
+    <row r="1" ht="18" customHeight="1" s="18">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>⚙️  HUTKO Kitchen — Contact &amp; Business Settings</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>Edit values in column B. These are read by the website for the contact page, footer, and delivery info.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="6" customHeight="1" s="17"/>
+    <row r="3" ht="6" customHeight="1" s="18"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -2529,7 +2530,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;"Calibri"&amp;10 &amp;KFF0000_x000d_# C2-Vertrouwelijk</oddFooter>
+    <oddFooter>&amp;C&amp;"Calibri"&amp;10 &amp;KFF0000_x000d_# C2-Vertrouwelijk_x000d_&amp;1#&amp;"Calibri"&amp;10 &amp;K008000 C0-Openbaar</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>